<commit_message>
Transformer sizing: 2/3 combinations, ratings input, standby groups, kW/kvar, Excel report
- Ratings typed in the UI (one or several); choose automatic, 2 or 3 transformers
- Per-combination distribution with duty/standby group kept on different sections
- One-transformer-out check per transformer (remaining units <= 90 %)
- kW (input), kvar and power factor shown; total kVA basis selectable
- Excel report with a switch for kW/kvar/pf and a sheet per combination
- Sample workbook gains a duty/standby group column and a standby pump pair

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017fNG5ZkrunawmtUXyCLSAu
</commit_message>
<xml_diff>
--- a/public/sample_load_list.xlsx
+++ b/public/sample_load_list.xlsx
@@ -421,14 +421,15 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E16"/>
+  <dimension ref="A1:F17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="34" customWidth="1" min="1" max="1"/>
+    <col width="36" customWidth="1" min="1" max="1"/>
     <col width="22" customWidth="1" min="2" max="2"/>
     <col width="16" customWidth="1" min="3" max="3"/>
     <col width="16" customWidth="1" min="4" max="4"/>
     <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="20" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -457,11 +458,16 @@
           <t>Voltage level (V)</t>
         </is>
       </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Duty/standby group</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Boiler feed water pump</t>
+          <t>Boiler feed water pump A (duty)</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -475,11 +481,16 @@
       <c r="E2" t="n">
         <v>433</v>
       </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>BFW</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Cooling water pump A</t>
+          <t>Boiler feed water pump B (standby)</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -488,16 +499,21 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>160</v>
+        <v>185</v>
       </c>
       <c r="E3" t="n">
         <v>433</v>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>BFW</t>
+        </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Cooling water pump B (standby)</t>
+          <t>Cooling water pump A (duty)</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -511,29 +527,39 @@
       <c r="E4" t="n">
         <v>433</v>
       </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>CWP</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>ID fan</t>
+          <t>Cooling water pump B (standby)</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>VFD</t>
+          <t>DOL</t>
         </is>
       </c>
       <c r="D5" t="n">
-        <v>250</v>
+        <v>160</v>
       </c>
       <c r="E5" t="n">
         <v>433</v>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>CWP</t>
+        </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>FD fan</t>
+          <t>ID fan</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -542,7 +568,7 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>200</v>
+        <v>250</v>
       </c>
       <c r="E6" t="n">
         <v>433</v>
@@ -551,16 +577,16 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Air compressor</t>
+          <t>FD fan</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>DOL</t>
+          <t>VFD</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>132</v>
+        <v>200</v>
       </c>
       <c r="E7" t="n">
         <v>433</v>
@@ -569,7 +595,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Conveyor 1</t>
+          <t>Air compressor</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -578,7 +604,7 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>90</v>
+        <v>132</v>
       </c>
       <c r="E8" t="n">
         <v>433</v>
@@ -587,16 +613,16 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Conveyor 2</t>
+          <t>Conveyor 1</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>VFD</t>
+          <t>DOL</t>
         </is>
       </c>
       <c r="D9" t="n">
-        <v>75</v>
+        <v>90</v>
       </c>
       <c r="E9" t="n">
         <v>433</v>
@@ -605,16 +631,16 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Crusher</t>
+          <t>Conveyor 2</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>DOL</t>
+          <t>VFD</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>315</v>
+        <v>75</v>
       </c>
       <c r="E10" t="n">
         <v>433</v>
@@ -623,7 +649,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Dosing pump (amps only)</t>
+          <t>Crusher</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -631,8 +657,8 @@
           <t>DOL</t>
         </is>
       </c>
-      <c r="C11" t="n">
-        <v>180</v>
+      <c r="D11" t="n">
+        <v>315</v>
       </c>
       <c r="E11" t="n">
         <v>433</v>
@@ -641,16 +667,16 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Booster fan (amps only)</t>
+          <t>Dosing pump (amps only)</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>VFD</t>
+          <t>DOL</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>120</v>
+        <v>180</v>
       </c>
       <c r="E12" t="n">
         <v>433</v>
@@ -659,16 +685,16 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Lighting &amp; small power DB</t>
+          <t>Booster fan (amps only)</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Feeder</t>
+          <t>VFD</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>250</v>
+        <v>120</v>
       </c>
       <c r="E13" t="n">
         <v>433</v>
@@ -677,7 +703,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>MCC-2 incomer</t>
+          <t>Lighting &amp; small power DB</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -686,7 +712,7 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>800</v>
+        <v>250</v>
       </c>
       <c r="E14" t="n">
         <v>433</v>
@@ -695,36 +721,54 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Grinding mill</t>
+          <t>MCC-2 incomer</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>DOL</t>
-        </is>
-      </c>
-      <c r="D15" t="n">
-        <v>450</v>
+          <t>Feeder</t>
+        </is>
+      </c>
+      <c r="C15" t="n">
+        <v>800</v>
       </c>
       <c r="E15" t="n">
-        <v>690</v>
+        <v>433</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
+          <t>Grinding mill</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>DOL</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>450</v>
+      </c>
+      <c r="E16" t="n">
+        <v>690</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
           <t>Slurry pump</t>
         </is>
       </c>
-      <c r="B16" t="inlineStr">
+      <c r="B17" t="inlineStr">
         <is>
           <t>VFD</t>
         </is>
       </c>
-      <c r="D16" t="n">
+      <c r="D17" t="n">
         <v>355</v>
       </c>
-      <c r="E16" t="n">
+      <c r="E17" t="n">
         <v>690</v>
       </c>
     </row>
@@ -739,7 +783,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A8"/>
+  <dimension ref="A1:A10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="110" customWidth="1" min="1" max="1"/>
@@ -797,6 +841,20 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
+          <t>Duty/standby group (optional): loads with the same group name are placed on different transformers' bus sections.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Optional columns can be left out; extra columns are ignored.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
           <t>The values in this file are examples only.</t>
         </is>
       </c>

</xml_diff>

<commit_message>
Transformer sizing: rating radio buttons, W/S column, fixed limits, arithmetic total
- Rating chosen with radio buttons (2000 / 2500 / 4000 kVA, default 2000); hint when the chosen rating does not fit
- Working/Standby (W/S) column read from the load list and shown in the GUI, distribution and Excel report
- 80 % / 90 % limits fixed; total kVA is the arithmetic sum only (vector option removed from the UI and report)
- Sample workbook gains a W/S column

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017fNG5ZkrunawmtUXyCLSAu
</commit_message>
<xml_diff>
--- a/public/sample_load_list.xlsx
+++ b/public/sample_load_list.xlsx
@@ -421,15 +421,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F17"/>
+  <dimension ref="A1:G17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="36" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="1" max="1"/>
     <col width="22" customWidth="1" min="2" max="2"/>
     <col width="16" customWidth="1" min="3" max="3"/>
     <col width="16" customWidth="1" min="4" max="4"/>
     <col width="16" customWidth="1" min="5" max="5"/>
-    <col width="20" customWidth="1" min="6" max="6"/>
+    <col width="22" customWidth="1" min="6" max="6"/>
+    <col width="20" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -460,6 +461,11 @@
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
+          <t>Working/Standby (W/S)</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
           <t>Duty/standby group</t>
         </is>
       </c>
@@ -467,7 +473,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Boiler feed water pump A (duty)</t>
+          <t>Boiler feed water pump A</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -483,6 +489,11 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
+          <t>W</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
           <t>BFW</t>
         </is>
       </c>
@@ -490,7 +501,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Boiler feed water pump B (standby)</t>
+          <t>Boiler feed water pump B</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -506,6 +517,11 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
           <t>BFW</t>
         </is>
       </c>
@@ -513,7 +529,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Cooling water pump A (duty)</t>
+          <t>Cooling water pump A</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -529,6 +545,11 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
+          <t>W</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
           <t>CWP</t>
         </is>
       </c>
@@ -536,7 +557,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Cooling water pump B (standby)</t>
+          <t>Cooling water pump B</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -552,6 +573,11 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
           <t>CWP</t>
         </is>
       </c>
@@ -573,6 +599,11 @@
       <c r="E6" t="n">
         <v>433</v>
       </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -591,6 +622,11 @@
       <c r="E7" t="n">
         <v>433</v>
       </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -609,6 +645,11 @@
       <c r="E8" t="n">
         <v>433</v>
       </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -627,6 +668,11 @@
       <c r="E9" t="n">
         <v>433</v>
       </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -645,6 +691,11 @@
       <c r="E10" t="n">
         <v>433</v>
       </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -663,6 +714,11 @@
       <c r="E11" t="n">
         <v>433</v>
       </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -681,6 +737,11 @@
       <c r="E12" t="n">
         <v>433</v>
       </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -699,6 +760,11 @@
       <c r="E13" t="n">
         <v>433</v>
       </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -717,6 +783,11 @@
       <c r="E14" t="n">
         <v>433</v>
       </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -735,6 +806,11 @@
       <c r="E15" t="n">
         <v>433</v>
       </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -753,6 +829,11 @@
       <c r="E16" t="n">
         <v>690</v>
       </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -770,6 +851,11 @@
       </c>
       <c r="E17" t="n">
         <v>690</v>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -783,7 +869,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A10"/>
+  <dimension ref="A1:A11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="110" customWidth="1" min="1" max="1"/>
@@ -841,19 +927,26 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Duty/standby group (optional): loads with the same group name are placed on different transformers' bus sections.</t>
+          <t>Working/Standby (optional): W = working, S = standby. Shown as W / S in the results. Standby loads are counted at 100 % like working loads.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Optional columns can be left out; extra columns are ignored.</t>
+          <t>Duty/standby group (optional): loads with the same group name are placed on different transformers' bus sections.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
+        <is>
+          <t>Optional columns can be left out; extra columns are ignored.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
         <is>
           <t>The values in this file are examples only.</t>
         </is>

</xml_diff>

<commit_message>
Current (A) column after kVA; replace the sample file with the supplied 29-row list
The supplied file had 'Bolier' again in one group and author metadata; both removed as before.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017fNG5ZkrunawmtUXyCLSAu
</commit_message>
<xml_diff>
--- a/public/sample_load_list.xlsx
+++ b/public/sample_load_list.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\1032578\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2503C7FB-84F6-4F1D-AEE3-49DB21004FB7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{350A4C91-C5D8-4CC1-86BD-836C94215E1C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Load list" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="87" uniqueCount="43">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="122" uniqueCount="54">
   <si>
     <t>Description</t>
   </si>
@@ -163,13 +163,46 @@
   </si>
   <si>
     <t>ESP</t>
+  </si>
+  <si>
+    <t>HGMS 2 Feed Pump 1</t>
+  </si>
+  <si>
+    <t>HGMS 2 Feed Pump 2</t>
+  </si>
+  <si>
+    <t>HGMS 2 Feed Pump 3</t>
+  </si>
+  <si>
+    <t>HGMS 2 Feed Pump 4</t>
+  </si>
+  <si>
+    <t>Warman slurry pump for Stirred Mill-1</t>
+  </si>
+  <si>
+    <t>HGMS 1 Feed Pump 1</t>
+  </si>
+  <si>
+    <t>HGMS 1 Feed Pump 2</t>
+  </si>
+  <si>
+    <t>HGMS 1 Feed Pump 3</t>
+  </si>
+  <si>
+    <t>HGMS 1 Feed Pump 4</t>
+  </si>
+  <si>
+    <t>HGMS2 Feed Pump</t>
+  </si>
+  <si>
+    <t>HGMS1 Feed Pump</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -181,6 +214,18 @@
       <b/>
       <sz val="11"/>
       <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
@@ -218,7 +263,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -233,6 +278,9 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -536,7 +584,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G21"/>
+  <dimension ref="A1:G30"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="36" customWidth="1"/>
@@ -969,7 +1017,195 @@
       </c>
       <c r="G21" s="6"/>
     </row>
+    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A22" s="7" t="s">
+        <v>43</v>
+      </c>
+      <c r="B22" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="C22" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="D22" s="6"/>
+      <c r="E22" s="6">
+        <v>250</v>
+      </c>
+      <c r="F22" s="6">
+        <v>433</v>
+      </c>
+      <c r="G22" s="6" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A23" s="7" t="s">
+        <v>44</v>
+      </c>
+      <c r="B23" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="C23" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="D23" s="6"/>
+      <c r="E23" s="6">
+        <v>250</v>
+      </c>
+      <c r="F23" s="6">
+        <v>433</v>
+      </c>
+      <c r="G23" s="6" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A24" s="7" t="s">
+        <v>45</v>
+      </c>
+      <c r="B24" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="C24" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="D24" s="6"/>
+      <c r="E24" s="6">
+        <v>250</v>
+      </c>
+      <c r="F24" s="6">
+        <v>433</v>
+      </c>
+      <c r="G24" s="6" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A25" s="7" t="s">
+        <v>46</v>
+      </c>
+      <c r="B25" s="6" t="s">
+        <v>39</v>
+      </c>
+      <c r="C25" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="D25" s="6"/>
+      <c r="E25" s="6">
+        <v>250</v>
+      </c>
+      <c r="F25" s="6">
+        <v>433</v>
+      </c>
+      <c r="G25" s="6" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A26" s="7" t="s">
+        <v>47</v>
+      </c>
+      <c r="B26" s="6" t="s">
+        <v>39</v>
+      </c>
+      <c r="C26" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="D26" s="6"/>
+      <c r="E26" s="6">
+        <v>110</v>
+      </c>
+      <c r="F26" s="6">
+        <v>433</v>
+      </c>
+      <c r="G26" s="6"/>
+    </row>
+    <row r="27" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A27" s="7" t="s">
+        <v>48</v>
+      </c>
+      <c r="B27" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="C27" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="D27" s="6"/>
+      <c r="E27" s="6">
+        <v>250</v>
+      </c>
+      <c r="F27" s="6">
+        <v>433</v>
+      </c>
+      <c r="G27" s="6" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A28" s="7" t="s">
+        <v>49</v>
+      </c>
+      <c r="B28" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="C28" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="D28" s="6"/>
+      <c r="E28" s="6">
+        <v>250</v>
+      </c>
+      <c r="F28" s="6">
+        <v>433</v>
+      </c>
+      <c r="G28" s="6" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="29" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A29" s="7" t="s">
+        <v>50</v>
+      </c>
+      <c r="B29" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="C29" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="D29" s="6"/>
+      <c r="E29" s="6">
+        <v>250</v>
+      </c>
+      <c r="F29" s="6">
+        <v>433</v>
+      </c>
+      <c r="G29" s="6" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="30" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A30" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="B30" s="6" t="s">
+        <v>39</v>
+      </c>
+      <c r="C30" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="D30" s="6"/>
+      <c r="E30" s="6">
+        <v>250</v>
+      </c>
+      <c r="F30" s="6">
+        <v>433</v>
+      </c>
+      <c r="G30" s="6" t="s">
+        <v>53</v>
+      </c>
+    </row>
   </sheetData>
+  <phoneticPr fontId="3" type="noConversion"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
New sample load list (40 rows); compact view; tests updated for the new sample
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017fNG5ZkrunawmtUXyCLSAu
</commit_message>
<xml_diff>
--- a/public/sample_load_list.xlsx
+++ b/public/sample_load_list.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\1032578\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{350A4C91-C5D8-4CC1-86BD-836C94215E1C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CFCC6DCA-1EC3-43D2-9677-A2A39DA72DEC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="122" uniqueCount="54">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="163" uniqueCount="67">
   <si>
     <t>Description</t>
   </si>
@@ -196,6 +196,45 @@
   </si>
   <si>
     <t>HGMS1 Feed Pump</t>
+  </si>
+  <si>
+    <t>Thickener 1 Feed Pump 1</t>
+  </si>
+  <si>
+    <t>Thickener1 Feed Pump</t>
+  </si>
+  <si>
+    <t>Thickener 1 Feed Pump 2</t>
+  </si>
+  <si>
+    <t>Thickener 1 Feed Pump 3</t>
+  </si>
+  <si>
+    <t>Thickener 1 Feed Pump 4</t>
+  </si>
+  <si>
+    <t>Thickener 2 Feed Pump 1</t>
+  </si>
+  <si>
+    <t>Thickener2 Feed Pump</t>
+  </si>
+  <si>
+    <t>Thickener 2 Feed Pump 2</t>
+  </si>
+  <si>
+    <t>Thickener 2 Feed Pump 3</t>
+  </si>
+  <si>
+    <t>Thickener 2 Feed Pump 4</t>
+  </si>
+  <si>
+    <t>MCC-3 incomer</t>
+  </si>
+  <si>
+    <t>MCC-4 incomer</t>
+  </si>
+  <si>
+    <t>MCC-5 incomer</t>
   </si>
 </sst>
 </file>
@@ -214,6 +253,7 @@
       <b/>
       <sz val="11"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="10"/>
@@ -584,14 +624,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G30"/>
+  <dimension ref="A1:G41"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="36" customWidth="1"/>
     <col min="2" max="2" width="4.85546875" style="2" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="22" style="2" customWidth="1"/>
     <col min="4" max="6" width="16" style="2" customWidth="1"/>
-    <col min="7" max="7" width="20" style="2" customWidth="1"/>
+    <col min="7" max="7" width="25.28515625" style="2" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="30" x14ac:dyDescent="0.25">
@@ -1203,6 +1243,231 @@
       <c r="G30" s="6" t="s">
         <v>53</v>
       </c>
+    </row>
+    <row r="31" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A31" s="7" t="s">
+        <v>54</v>
+      </c>
+      <c r="B31" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="C31" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="D31" s="6"/>
+      <c r="E31" s="6">
+        <v>200</v>
+      </c>
+      <c r="F31" s="6">
+        <v>433</v>
+      </c>
+      <c r="G31" s="6" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="32" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A32" s="7" t="s">
+        <v>56</v>
+      </c>
+      <c r="B32" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="C32" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="D32" s="6"/>
+      <c r="E32" s="6">
+        <v>200</v>
+      </c>
+      <c r="F32" s="6">
+        <v>433</v>
+      </c>
+      <c r="G32" s="6" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="33" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A33" s="7" t="s">
+        <v>57</v>
+      </c>
+      <c r="B33" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="C33" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="D33" s="6"/>
+      <c r="E33" s="6">
+        <v>200</v>
+      </c>
+      <c r="F33" s="6">
+        <v>433</v>
+      </c>
+      <c r="G33" s="6" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="34" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A34" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="B34" s="6" t="s">
+        <v>39</v>
+      </c>
+      <c r="C34" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="D34" s="6"/>
+      <c r="E34" s="6">
+        <v>200</v>
+      </c>
+      <c r="F34" s="6">
+        <v>433</v>
+      </c>
+      <c r="G34" s="6" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="35" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A35" s="7" t="s">
+        <v>59</v>
+      </c>
+      <c r="B35" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="C35" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="D35" s="6"/>
+      <c r="E35" s="6">
+        <v>275</v>
+      </c>
+      <c r="F35" s="6">
+        <v>433</v>
+      </c>
+      <c r="G35" s="6" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="36" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A36" s="7" t="s">
+        <v>61</v>
+      </c>
+      <c r="B36" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="C36" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="D36" s="6"/>
+      <c r="E36" s="6">
+        <v>275</v>
+      </c>
+      <c r="F36" s="6">
+        <v>433</v>
+      </c>
+      <c r="G36" s="6" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="37" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A37" s="7" t="s">
+        <v>62</v>
+      </c>
+      <c r="B37" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="C37" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="D37" s="6"/>
+      <c r="E37" s="6">
+        <v>275</v>
+      </c>
+      <c r="F37" s="6">
+        <v>433</v>
+      </c>
+      <c r="G37" s="6" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="38" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A38" s="7" t="s">
+        <v>63</v>
+      </c>
+      <c r="B38" s="6" t="s">
+        <v>39</v>
+      </c>
+      <c r="C38" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="D38" s="6"/>
+      <c r="E38" s="6">
+        <v>275</v>
+      </c>
+      <c r="F38" s="6">
+        <v>433</v>
+      </c>
+      <c r="G38" s="6" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="39" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A39" s="5" t="s">
+        <v>64</v>
+      </c>
+      <c r="B39" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="C39" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="D39" s="6">
+        <v>550</v>
+      </c>
+      <c r="E39" s="6"/>
+      <c r="F39" s="6">
+        <v>433</v>
+      </c>
+      <c r="G39" s="6"/>
+    </row>
+    <row r="40" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A40" s="5" t="s">
+        <v>65</v>
+      </c>
+      <c r="B40" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="C40" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="D40" s="6">
+        <v>700</v>
+      </c>
+      <c r="E40" s="6"/>
+      <c r="F40" s="6">
+        <v>433</v>
+      </c>
+      <c r="G40" s="6"/>
+    </row>
+    <row r="41" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A41" s="5" t="s">
+        <v>66</v>
+      </c>
+      <c r="B41" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="C41" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="D41" s="6">
+        <v>900</v>
+      </c>
+      <c r="E41" s="6"/>
+      <c r="F41" s="6">
+        <v>433</v>
+      </c>
+      <c r="G41" s="6"/>
     </row>
   </sheetData>
   <phoneticPr fontId="3" type="noConversion"/>

</xml_diff>